<commit_message>
fix(pipeline): deduplicar observaciones trimestrales y completar EMOE/BCMM
- Corrige apply_inegi_total para colapsar observaciones de series
  trimestrales del INEGI que se publican con múltiples TIME_PERIOD
  mensuales dentro del mismo trimestre, evitando duplicados en PIB
  y PIBSEC.
- Agrega series oficiales de EMOE (confianza + variación) y BCMM
  (exportaciones + importaciones) con saldo derivado.
- Ajusta la lógica de frescura para series agregadas diarias/semanales
  a mensuales (RESERVAS, TASA, TIPOCAMBIO).
- Carga 2T-26 P del PIB con variaciones del EOPIBT y marca el nivel
  como pendiente de publicación.
- Actualiza tests y datos generados (CSV, Excel, JSON).

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/CONSUMO/CONSUMO_datos.xlsx
+++ b/downloads/indicadores/CONSUMO/CONSUMO_datos.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -577,14 +577,14 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Nov 24</t>
+          <t>Oct 24</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>45597</v>
+        <v>45566</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>111</v>
+        <v>110.5</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -635,18 +635,18 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Dic 24</t>
+          <t>Nov 24</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>45627</v>
+        <v>45597</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>109.4</v>
+        <v>111</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-1.1%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-0.8%</t>
+          <t>+0.7%</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -693,18 +693,18 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Ene 25</t>
+          <t>Dic 24</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>45658</v>
+        <v>45627</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>108.6</v>
+        <v>109.4</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-0.3%</t>
+          <t>-1.1%</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>-0.9%</t>
+          <t>-0.8%</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -751,18 +751,18 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Feb 25</t>
+          <t>Ene 25</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>45689</v>
+        <v>45658</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>110.2</v>
+        <v>108.6</v>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>-0.3%</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>-0.7%</t>
+          <t>-0.9%</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -809,18 +809,18 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Mar 25</t>
+          <t>Feb 25</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>45717</v>
+        <v>45689</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>110.2</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>-0.2%</t>
+          <t>+1.2%</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>-1.3%</t>
+          <t>-0.7%</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -867,18 +867,18 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Abr 25 R</t>
+          <t>Mar 25</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>45748</v>
+        <v>45717</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>111.6</v>
+        <v>110.2</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>+1.1%</t>
+          <t>-0.2%</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>+0.7%</t>
+          <t>-1.3%</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Revisado</t>
+          <t>Definitivo</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -925,18 +925,18 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>May 25 R</t>
+          <t>Abr 25 R</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>45778</v>
+        <v>45748</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>110.1</v>
+        <v>111.6</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>-1.0%</t>
+          <t>+1.1%</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>-0.9%</t>
+          <t>+0.7%</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -983,18 +983,18 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Jun 25 R</t>
+          <t>May 25 R</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>45809</v>
+        <v>45778</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>111.5</v>
+        <v>110.1</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>+0.8%</t>
+          <t>-1.0%</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>+1.1%</t>
+          <t>-0.9%</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1041,18 +1041,18 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Jul 25 R</t>
+          <t>Jun 25 R</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>45839</v>
+        <v>45809</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>111.2</v>
+        <v>111.5</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>-0.3%</t>
+          <t>+0.8%</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>-0.1%</t>
+          <t>+1.1%</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1099,18 +1099,18 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Ago 25 R</t>
+          <t>Jul 25 R</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>45870</v>
+        <v>45839</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>112.1</v>
+        <v>111.2</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>+0.6%</t>
+          <t>-0.3%</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>+0.9%</t>
+          <t>-0.1%</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1157,18 +1157,18 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Sep 25 R</t>
+          <t>Ago 25 R</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>45901</v>
+        <v>45870</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>112.4</v>
+        <v>112.1</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>+0.6%</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>+2.1%</t>
+          <t>+0.9%</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1215,18 +1215,18 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Oct 25 R</t>
+          <t>Sep 25 R</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>45931</v>
+        <v>45901</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>113.5</v>
+        <v>112.4</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>+0.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>+4.1%</t>
+          <t>+2.1%</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1273,18 +1273,18 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Nov 25 R</t>
+          <t>Oct 25 R</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>45962</v>
+        <v>45931</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>112.9</v>
+        <v>113.5</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>-0.5%</t>
+          <t>+0.8%</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>+2.8%</t>
+          <t>+4.1%</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1331,18 +1331,18 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Dic 25 R</t>
+          <t>Nov 25 R</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>45992</v>
+        <v>45962</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>114.4</v>
+        <v>112.9</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>-0.5%</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>+5.6%</t>
+          <t>+2.8%</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1389,18 +1389,18 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Ene 26 R</t>
+          <t>Dic 25 R</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>46023</v>
+        <v>45992</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>112.1</v>
+        <v>114.4</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>-1.6%</t>
+          <t>+1.2%</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>+2.7%</t>
+          <t>+5.6%</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1447,18 +1447,18 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Feb 26 R</t>
+          <t>Ene 26 R</t>
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>46054</v>
+        <v>46023</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>111.4</v>
+        <v>112.1</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>-0.5%</t>
+          <t>-1.6%</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>+0.9%</t>
+          <t>+2.7%</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1505,18 +1505,18 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Mar 26 P</t>
+          <t>Feb 26 R</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>46082</v>
+        <v>46054</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>113.6</v>
+        <v>111.4</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>-0.5%</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>+3.1%</t>
+          <t>+0.9%</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Preliminar</t>
+          <t>Revisado</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1563,18 +1563,18 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Abr 26</t>
+          <t>Mar 26 P</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>46113</v>
+        <v>46082</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>113.7</v>
+        <v>113.6</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>+1.2%</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>+2.1%</t>
+          <t>+3.1%</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>Definitivo</t>
+          <t>Preliminar</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
@@ -1621,56 +1621,114 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>Abr 26</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>46113</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>113.7</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>+0.1%</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>+2.1%</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Índice base 2018=100</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Serie desestacionalizada; índice y variaciones oficiales del boletín del INEGI</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Definitivo</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>INEGI</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/imcp/imcpmi2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>05 de agosto de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
           <t>May 26</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B25" s="8" t="n">
         <v>46143</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C25" s="9" t="n">
         <v>114</v>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>+0.1%</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>+2.6%</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Índice base 2018=100</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Serie desestacionalizada; índice y variaciones oficiales del boletín del INEGI</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Índice base 2018=100</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Serie desestacionalizada; índice y variaciones oficiales del boletín del INEGI</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>INEGI</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/imcp/imcpmi2026_08.pdf</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>INEGI</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/imcp/imcpmi2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
         <is>
           <t>05 de agosto de 2026</t>
         </is>

</xml_diff>